<commit_message>
abbruchkriterien PSO und cost-erstellung
</commit_message>
<xml_diff>
--- a/PlayGround/Verification Freq_Metrics low_constraints/Referenzsysteme.xlsx
+++ b/PlayGround/Verification Freq_Metrics low_constraints/Referenzsysteme.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Flo\Datenbox9000\ZHAW\Faecher\BA\Control-Optimizer\PlayGround\Verification Freq_Metrics low_constraints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322F527B-5278-4DEF-AB0A-BE6D864014AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B02CBA-50D8-494E-93F3-50F96C8860B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BF42E3A3-33EF-4DBC-9F5E-81167A7AA33A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
   <si>
     <t>PTn</t>
   </si>
@@ -71,10 +71,16 @@
     <t>aus PA</t>
   </si>
   <si>
-    <t>diff</t>
+    <t>low constraints V1</t>
   </si>
   <si>
-    <t>low constraints</t>
+    <t>diff V1</t>
+  </si>
+  <si>
+    <t>low constraints V2</t>
+  </si>
+  <si>
+    <t>diff V2</t>
   </si>
 </sst>
 </file>
@@ -90,18 +96,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -116,9 +116,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -453,15 +452,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCA6B1ED-5E04-4CAB-9D93-436689B1170E}">
-  <dimension ref="A2:J66"/>
+  <dimension ref="A2:M66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="8" width="16" customWidth="1"/>
-    <col min="10" max="10" width="19.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="19.7109375" customWidth="1"/>
     <col min="18" max="18" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -469,10 +469,19 @@
         <v>10</v>
       </c>
       <c r="H2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -494,11 +503,8 @@
       <c r="G3" t="s">
         <v>6</v>
       </c>
-      <c r="J3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -523,12 +529,19 @@
       <c r="H4">
         <v>7.1095818636902633E-2</v>
       </c>
-      <c r="J4">
-        <f>G4-H4</f>
+      <c r="I4">
+        <v>7.8190068006843194E-2</v>
+      </c>
+      <c r="L4">
+        <f t="shared" ref="L4:L27" si="0">G4-H4</f>
         <v>-8.1520275842403289E-4</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M4">
+        <f>G4-I4</f>
+        <v>-7.9094521283645941E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -553,12 +566,19 @@
       <c r="H5">
         <v>3.041755473293923E-2</v>
       </c>
-      <c r="J5">
-        <f t="shared" ref="J5:J66" si="0">G5-H5</f>
+      <c r="I5">
+        <v>3.0129294364536981E-2</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="0"/>
         <v>-1.1925637367898312E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M5">
+        <f t="shared" ref="M5:M66" si="1">G5-I5</f>
+        <v>-9.0430336838758299E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -583,12 +603,19 @@
       <c r="H6">
         <v>1.380102902752884E-2</v>
       </c>
-      <c r="J6">
+      <c r="I6">
+        <v>1.374002847187117E-2</v>
+      </c>
+      <c r="L6">
         <f t="shared" si="0"/>
         <v>9.6668583345598663E-6</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M6">
+        <f t="shared" si="1"/>
+        <v>7.0667413992229339E-5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -613,12 +640,19 @@
       <c r="H7">
         <v>1.012176056726889E-2</v>
       </c>
-      <c r="J7">
+      <c r="I7">
+        <v>9.9811297553203705E-3</v>
+      </c>
+      <c r="L7">
         <f t="shared" si="0"/>
         <v>-1.1945975227229018E-4</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M7">
+        <f t="shared" si="1"/>
+        <v>2.117105967622962E-5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
@@ -643,12 +677,19 @@
       <c r="H8">
         <v>0.59156538673460868</v>
       </c>
-      <c r="J8">
+      <c r="I8">
+        <v>0.5903456723861441</v>
+      </c>
+      <c r="L8">
         <f t="shared" si="0"/>
         <v>1.7242854069062785E-3</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M8">
+        <f t="shared" si="1"/>
+        <v>2.9439997553708519E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2</v>
       </c>
@@ -673,12 +714,19 @@
       <c r="H9">
         <v>0.3620639610069521</v>
       </c>
-      <c r="J9">
+      <c r="I9">
+        <v>0.36248705785893309</v>
+      </c>
+      <c r="L9">
         <f t="shared" si="0"/>
         <v>3.2536505510988301E-4</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M9">
+        <f t="shared" si="1"/>
+        <v>-9.773179687111444E-5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2</v>
       </c>
@@ -703,12 +751,19 @@
       <c r="H10">
         <v>0.2388612525349979</v>
       </c>
-      <c r="J10">
+      <c r="I10">
+        <v>0.23831659469907121</v>
+      </c>
+      <c r="L10">
         <f t="shared" si="0"/>
         <v>2.7850728929310065E-4</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M10">
+        <f t="shared" si="1"/>
+        <v>8.2316512521979357E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -733,12 +788,19 @@
       <c r="H11">
         <v>0.18779180065763121</v>
       </c>
-      <c r="J11">
+      <c r="I11">
+        <v>0.18726141601148041</v>
+      </c>
+      <c r="L11">
         <f t="shared" si="0"/>
         <v>-1.3533519483022172E-4</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M11">
+        <f t="shared" si="1"/>
+        <v>3.9504945132057268E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>3</v>
       </c>
@@ -763,12 +825,19 @@
       <c r="H12">
         <v>1.871422016624041</v>
       </c>
-      <c r="J12">
+      <c r="I12">
+        <v>1.8656588572473241</v>
+      </c>
+      <c r="L12">
         <f t="shared" si="0"/>
         <v>-6.3593083177908571E-3</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M12">
+        <f t="shared" si="1"/>
+        <v>-5.9614894107395955E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>3</v>
       </c>
@@ -793,12 +862,19 @@
       <c r="H13">
         <v>1.3437579083176221</v>
       </c>
-      <c r="J13">
+      <c r="I13">
+        <v>1.343304146520534</v>
+      </c>
+      <c r="L13">
         <f t="shared" si="0"/>
         <v>1.350169433578241E-4</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M13">
+        <f t="shared" si="1"/>
+        <v>5.8877874044593881E-4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>3</v>
       </c>
@@ -823,12 +899,19 @@
       <c r="H14">
         <v>1.005784746332927</v>
       </c>
-      <c r="J14">
+      <c r="I14">
+        <v>1.0056609393882321</v>
+      </c>
+      <c r="L14">
         <f t="shared" si="0"/>
         <v>4.2738297817290771E-4</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M14">
+        <f t="shared" si="1"/>
+        <v>5.5118992286784518E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>3</v>
       </c>
@@ -853,377 +936,468 @@
       <c r="H15">
         <v>0.80307011280353224</v>
       </c>
-      <c r="J15">
+      <c r="I15">
+        <v>0.80374909931423755</v>
+      </c>
+      <c r="L15">
         <f t="shared" si="0"/>
         <v>1.8959548600907539E-3</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+      <c r="M15">
+        <f t="shared" si="1"/>
+        <v>1.21696834938545E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>4</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16">
         <v>-2</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16">
         <v>2</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16">
         <v>1.9141764468840201</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16">
         <v>5.0469723397912203</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16">
         <v>1.1118171071037299</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16">
         <v>4.7094791191536398</v>
       </c>
       <c r="H16">
         <v>4.7091672876219963</v>
       </c>
-      <c r="J16">
+      <c r="I16">
+        <v>4.7091183883263614</v>
+      </c>
+      <c r="L16">
         <f t="shared" si="0"/>
         <v>3.1183153164349164E-4</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
+      <c r="M16">
+        <f t="shared" si="1"/>
+        <v>3.6073082727838823E-4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>4</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17">
         <v>-3</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17">
         <v>3</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17">
         <v>2.3040036519432299</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17">
         <v>5.66275235588855</v>
       </c>
-      <c r="F17" s="1">
+      <c r="F17">
         <v>1.1758577109277399</v>
       </c>
-      <c r="G17" s="1">
+      <c r="G17">
         <v>4.4935715744873796</v>
       </c>
       <c r="H17">
         <v>4.4937452609668984</v>
       </c>
-      <c r="J17">
+      <c r="I17">
+        <v>4.4935163964116844</v>
+      </c>
+      <c r="L17">
         <f t="shared" si="0"/>
         <v>-1.7368647951876426E-4</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
+      <c r="M17">
+        <f t="shared" si="1"/>
+        <v>5.5178075695216933E-5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>4</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18">
         <v>-5</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18">
         <v>5</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18">
         <v>2.2714519236097699</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18">
         <v>5.51935642913761</v>
       </c>
-      <c r="F18" s="1">
+      <c r="F18">
         <v>1.1653828129892401</v>
       </c>
-      <c r="G18" s="1">
+      <c r="G18">
         <v>4.3951716448785998</v>
       </c>
       <c r="H18">
         <v>4.3949642719873498</v>
       </c>
-      <c r="J18">
+      <c r="I18">
+        <v>4.3950485632120104</v>
+      </c>
+      <c r="L18">
         <f t="shared" si="0"/>
         <v>2.0737289124994618E-4</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
+      <c r="M18">
+        <f t="shared" si="1"/>
+        <v>1.2308166658936415E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>4</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19">
         <v>-10</v>
       </c>
-      <c r="C19" s="1">
-        <v>10</v>
-      </c>
-      <c r="D19" s="1">
+      <c r="C19">
+        <v>10</v>
+      </c>
+      <c r="D19">
         <v>2.24378148402453</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19">
         <v>5.3006034470239296</v>
       </c>
-      <c r="F19" s="1">
+      <c r="F19">
         <v>1.1532169082485</v>
       </c>
-      <c r="G19" s="1">
+      <c r="G19">
         <v>4.2129653443995503</v>
       </c>
       <c r="H19">
         <v>4.2133239221670822</v>
       </c>
-      <c r="J19">
+      <c r="I19">
+        <v>4.2129355652907137</v>
+      </c>
+      <c r="L19">
         <f t="shared" si="0"/>
         <v>-3.5857776753189796E-4</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
+      <c r="M19">
+        <f t="shared" si="1"/>
+        <v>2.9779108836613943E-5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>5</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20">
         <v>-2</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20">
         <v>2</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20">
         <v>1.42656051809038</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20">
         <v>5.2741020018329801</v>
       </c>
-      <c r="F20" s="1">
+      <c r="F20">
         <v>1.46068019588464</v>
       </c>
-      <c r="G20" s="1">
+      <c r="G20">
         <v>9.8260517694073304</v>
       </c>
       <c r="H20">
         <v>9.8259374380106355</v>
       </c>
-      <c r="J20">
+      <c r="I20">
+        <v>9.8264365819680766</v>
+      </c>
+      <c r="L20">
         <f t="shared" si="0"/>
         <v>1.143313966949222E-4</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
+      <c r="M20">
+        <f t="shared" si="1"/>
+        <v>-3.8481256074618386E-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>5</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21">
         <v>-3</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21">
         <v>3</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21">
         <v>1.42202141153204</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21">
         <v>5.2287260417778301</v>
       </c>
-      <c r="F21" s="1">
+      <c r="F21">
         <v>1.45813563590267</v>
       </c>
-      <c r="G21" s="1">
+      <c r="G21">
         <v>9.7003630222173491</v>
       </c>
       <c r="H21">
         <v>9.7002221836905811</v>
       </c>
-      <c r="J21">
+      <c r="I21">
+        <v>9.700669815274555</v>
+      </c>
+      <c r="L21">
         <f t="shared" si="0"/>
         <v>1.4083852676805009E-4</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
+      <c r="M21">
+        <f t="shared" si="1"/>
+        <v>-3.0679305720582306E-4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>5</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22">
         <v>-5</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22">
         <v>5</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22">
         <v>1.42049436599645</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22">
         <v>5.1501044401101801</v>
       </c>
-      <c r="F22" s="1">
+      <c r="F22">
         <v>1.4479149355905601</v>
       </c>
-      <c r="G22" s="1">
+      <c r="G22">
         <v>9.4952496649515297</v>
       </c>
       <c r="H22">
         <v>9.4959111758085104</v>
       </c>
-      <c r="J22">
+      <c r="I22">
+        <v>9.4958866218927653</v>
+      </c>
+      <c r="L22">
         <f t="shared" si="0"/>
         <v>-6.6151085698074041E-4</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
+      <c r="M22">
+        <f t="shared" si="1"/>
+        <v>-6.3695694123566682E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>5</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23">
         <v>-10</v>
       </c>
-      <c r="C23" s="1">
-        <v>10</v>
-      </c>
-      <c r="D23" s="1">
+      <c r="C23">
+        <v>10</v>
+      </c>
+      <c r="D23">
         <v>1.4048109084261</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23">
         <v>4.98269963934474</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F23">
         <v>1.4252557958506</v>
       </c>
-      <c r="G23" s="1">
+      <c r="G23">
         <v>9.0995914438217707</v>
       </c>
       <c r="H23">
         <v>9.0991845559607096</v>
       </c>
-      <c r="J23">
+      <c r="I23">
+        <v>9.0991865758876767</v>
+      </c>
+      <c r="L23">
         <f t="shared" si="0"/>
         <v>4.068878610610227E-4</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
+      <c r="M23">
+        <f t="shared" si="1"/>
+        <v>4.0486793409399979E-4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>6</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24">
         <v>-2</v>
       </c>
-      <c r="C24" s="1">
+      <c r="C24">
         <v>2</v>
       </c>
-      <c r="D24" s="1">
+      <c r="D24">
         <v>1.03945799283177</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24">
         <v>5.1434342064424898</v>
       </c>
-      <c r="F24" s="1">
+      <c r="F24">
         <v>1.6532360059141999</v>
       </c>
-      <c r="G24" s="1">
+      <c r="G24">
         <v>16.603264930804301</v>
       </c>
       <c r="H24">
         <v>16.602644462615991</v>
       </c>
-      <c r="J24">
+      <c r="I24">
+        <v>16.602817349507198</v>
+      </c>
+      <c r="L24">
         <f t="shared" si="0"/>
         <v>6.2046818830907569E-4</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
+      <c r="M24">
+        <f t="shared" si="1"/>
+        <v>4.4758129710231742E-4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>6</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25">
         <v>-3</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25">
         <v>3</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25">
         <v>1.0420461439136699</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25">
         <v>5.1214197351197104</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25">
         <v>1.64316354722427</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25">
         <v>16.403879681171301</v>
       </c>
       <c r="H25">
         <v>16.403449432375741</v>
       </c>
-      <c r="J25">
+      <c r="I25">
+        <v>16.402795882113111</v>
+      </c>
+      <c r="L25">
         <f t="shared" si="0"/>
         <v>4.3024879555986217E-4</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
+      <c r="M25">
+        <f t="shared" si="1"/>
+        <v>1.0837990581897827E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>6</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26">
         <v>-5</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26">
         <v>5</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26">
         <v>1.03901518704408</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26">
         <v>5.0584309313238398</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26">
         <v>1.64104601378253</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G26">
         <v>16.069345158962999</v>
       </c>
       <c r="H26">
         <v>16.06740095497004</v>
       </c>
-      <c r="J26">
+      <c r="I26">
+        <v>16.06797577395913</v>
+      </c>
+      <c r="L26">
         <f t="shared" si="0"/>
         <v>1.9442039929593591E-3</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
+      <c r="M26">
+        <f t="shared" si="1"/>
+        <v>1.3693850038691835E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>6</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27">
         <v>-10</v>
       </c>
-      <c r="C27" s="1">
-        <v>10</v>
-      </c>
-      <c r="D27" s="1">
+      <c r="C27">
+        <v>10</v>
+      </c>
+      <c r="D27">
         <v>1.0402192763078999</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27">
         <v>4.9421370174902401</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F27">
         <v>1.6188015918738199</v>
       </c>
-      <c r="G27" s="1">
+      <c r="G27">
         <v>15.4099635909299</v>
       </c>
       <c r="H27">
         <v>15.40741611363795</v>
       </c>
-      <c r="J27">
+      <c r="I27">
+        <v>15.40709064832585</v>
+      </c>
+      <c r="L27">
         <f t="shared" si="0"/>
         <v>2.5474772919498179E-3</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M27">
+        <f t="shared" si="1"/>
+        <v>2.8729426040499106E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1246,7 +1420,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1</v>
       </c>
@@ -1271,12 +1445,19 @@
       <c r="H31">
         <v>0.59262551271087527</v>
       </c>
-      <c r="J31">
-        <f t="shared" si="0"/>
+      <c r="I31">
+        <v>0.59063818829592563</v>
+      </c>
+      <c r="L31">
+        <f t="shared" ref="L31:L66" si="2">G31-H31</f>
         <v>-4.3446771087529701E-4</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M31">
+        <f t="shared" si="1"/>
+        <v>1.5528567040743457E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1</v>
       </c>
@@ -1301,12 +1482,19 @@
       <c r="H32">
         <v>0.3624350918176758</v>
       </c>
-      <c r="J32">
-        <f t="shared" si="0"/>
+      <c r="I32">
+        <v>0.36226297620630532</v>
+      </c>
+      <c r="L32">
+        <f t="shared" si="2"/>
         <v>-3.4125881767582689E-4</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M32">
+        <f t="shared" si="1"/>
+        <v>-1.6914320630534441E-4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1</v>
       </c>
@@ -1331,12 +1519,19 @@
       <c r="H33">
         <v>0.23902305683439951</v>
       </c>
-      <c r="J33">
-        <f t="shared" si="0"/>
+      <c r="I33">
+        <v>0.2376217926739152</v>
+      </c>
+      <c r="L33">
+        <f t="shared" si="2"/>
         <v>2.0659961656004922E-3</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M33">
+        <f t="shared" si="1"/>
+        <v>3.4672603260847978E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>1</v>
       </c>
@@ -1361,12 +1556,19 @@
       <c r="H34">
         <v>0.18742485501066661</v>
       </c>
-      <c r="J34">
-        <f t="shared" si="0"/>
+      <c r="I34">
+        <v>0.18802743651980541</v>
+      </c>
+      <c r="L34">
+        <f t="shared" si="2"/>
         <v>6.9298933338957092E-7</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M34">
+        <f t="shared" si="1"/>
+        <v>-6.018885198054158E-4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>0.7</v>
       </c>
@@ -1391,12 +1593,19 @@
       <c r="H35">
         <v>0.48562631926204569</v>
       </c>
-      <c r="J35">
-        <f t="shared" si="0"/>
+      <c r="I35">
+        <v>0.48554757464014697</v>
+      </c>
+      <c r="L35">
+        <f t="shared" si="2"/>
         <v>1.3863897379542967E-3</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M35">
+        <f t="shared" si="1"/>
+        <v>1.4651343598530153E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>0.7</v>
       </c>
@@ -1421,12 +1630,19 @@
       <c r="H36">
         <v>0.32283930397507588</v>
       </c>
-      <c r="J36">
-        <f t="shared" si="0"/>
+      <c r="I36">
+        <v>0.32291151272595209</v>
+      </c>
+      <c r="L36">
+        <f t="shared" si="2"/>
         <v>1.8652740249241462E-3</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M36">
+        <f t="shared" si="1"/>
+        <v>1.7930652740479336E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>0.7</v>
       </c>
@@ -1451,12 +1667,19 @@
       <c r="H37">
         <v>0.22636043510528431</v>
       </c>
-      <c r="J37">
-        <f t="shared" si="0"/>
+      <c r="I37">
+        <v>0.2256430102728425</v>
+      </c>
+      <c r="L37">
+        <f t="shared" si="2"/>
         <v>1.6963628947156972E-3</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M37">
+        <f t="shared" si="1"/>
+        <v>2.4137877271575015E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>0.7</v>
       </c>
@@ -1481,12 +1704,19 @@
       <c r="H38">
         <v>0.18159352714874319</v>
       </c>
-      <c r="J38">
-        <f t="shared" si="0"/>
+      <c r="I38">
+        <v>0.1815579390502898</v>
+      </c>
+      <c r="L38">
+        <f t="shared" si="2"/>
         <v>4.1206368512567981E-3</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M38">
+        <f t="shared" si="1"/>
+        <v>4.1562249497101855E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>0.6</v>
       </c>
@@ -1511,12 +1741,19 @@
       <c r="H39">
         <v>0.45747140403544928</v>
       </c>
-      <c r="J39">
-        <f t="shared" si="0"/>
+      <c r="I39">
+        <v>0.45754632850607813</v>
+      </c>
+      <c r="L39">
+        <f t="shared" si="2"/>
         <v>2.5429119645506981E-3</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M39">
+        <f t="shared" si="1"/>
+        <v>2.4679874939218527E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>0.6</v>
       </c>
@@ -1541,12 +1778,19 @@
       <c r="H40">
         <v>0.31200418645630468</v>
       </c>
-      <c r="J40">
-        <f t="shared" si="0"/>
+      <c r="I40">
+        <v>0.31304650444252541</v>
+      </c>
+      <c r="L40">
+        <f t="shared" si="2"/>
         <v>2.2442275436952985E-3</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M40">
+        <f t="shared" si="1"/>
+        <v>1.2019095574745675E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>0.6</v>
       </c>
@@ -1571,12 +1815,19 @@
       <c r="H41">
         <v>0.22167012541540751</v>
       </c>
-      <c r="J41">
-        <f t="shared" si="0"/>
+      <c r="I41">
+        <v>0.2217817038534384</v>
+      </c>
+      <c r="L41">
+        <f t="shared" si="2"/>
         <v>4.4415095845924957E-3</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M41">
+        <f t="shared" si="1"/>
+        <v>4.3299311465616053E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>0.6</v>
       </c>
@@ -1601,12 +1852,19 @@
       <c r="H42">
         <v>0.17772830745026999</v>
       </c>
-      <c r="J42">
-        <f t="shared" si="0"/>
+      <c r="I42">
+        <v>0.177831234190273</v>
+      </c>
+      <c r="L42">
+        <f t="shared" si="2"/>
         <v>7.4566185497300097E-3</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M42">
+        <f t="shared" si="1"/>
+        <v>7.3536918097270032E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>0.5</v>
       </c>
@@ -1631,12 +1889,19 @@
       <c r="H43">
         <v>0.43269708176080629</v>
       </c>
-      <c r="J43">
-        <f t="shared" si="0"/>
+      <c r="I43">
+        <v>0.43280172632298952</v>
+      </c>
+      <c r="L43">
+        <f t="shared" si="2"/>
         <v>4.3912862391937146E-3</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M43">
+        <f t="shared" si="1"/>
+        <v>4.2866416770104832E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>0.5</v>
       </c>
@@ -1661,12 +1926,19 @@
       <c r="H44">
         <v>0.30135141319110159</v>
       </c>
-      <c r="J44">
-        <f t="shared" si="0"/>
+      <c r="I44">
+        <v>0.30176307335777669</v>
+      </c>
+      <c r="L44">
+        <f t="shared" si="2"/>
         <v>6.6532438088984236E-3</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M44">
+        <f t="shared" si="1"/>
+        <v>6.2415836422233251E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>0.5</v>
       </c>
@@ -1691,12 +1963,19 @@
       <c r="H45">
         <v>0.21752382845568899</v>
       </c>
-      <c r="J45">
-        <f t="shared" si="0"/>
+      <c r="I45">
+        <v>0.2170245351877565</v>
+      </c>
+      <c r="L45">
+        <f t="shared" si="2"/>
         <v>5.393738544311022E-3</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M45">
+        <f t="shared" si="1"/>
+        <v>5.8930318122435155E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>0.5</v>
       </c>
@@ -1721,12 +2000,19 @@
       <c r="H46">
         <v>0.17258532927152481</v>
       </c>
-      <c r="J46">
-        <f t="shared" si="0"/>
+      <c r="I46">
+        <v>0.17419686166888271</v>
+      </c>
+      <c r="L46">
+        <f t="shared" si="2"/>
         <v>1.3402122728475185E-2</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M46">
+        <f t="shared" si="1"/>
+        <v>1.179059033111729E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>0.4</v>
       </c>
@@ -1751,12 +2037,19 @@
       <c r="H47">
         <v>0.40996579846792619</v>
       </c>
-      <c r="J47">
-        <f t="shared" si="0"/>
+      <c r="I47">
+        <v>0.41310512166355912</v>
+      </c>
+      <c r="L47">
+        <f t="shared" si="2"/>
         <v>6.0199105320737911E-3</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M47">
+        <f t="shared" si="1"/>
+        <v>2.8805873364408652E-3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>0.4</v>
       </c>
@@ -1781,12 +2074,19 @@
       <c r="H48">
         <v>0.28971045726644612</v>
       </c>
-      <c r="J48">
-        <f t="shared" si="0"/>
+      <c r="I48">
+        <v>0.29067276837793737</v>
+      </c>
+      <c r="L48">
+        <f t="shared" si="2"/>
         <v>7.7521797335538545E-3</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M48">
+        <f t="shared" si="1"/>
+        <v>6.7898686220626003E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>0.4</v>
       </c>
@@ -1811,12 +2111,19 @@
       <c r="H49">
         <v>0.21121819174078441</v>
       </c>
-      <c r="J49">
-        <f t="shared" si="0"/>
+      <c r="I49">
+        <v>0.21114213139093929</v>
+      </c>
+      <c r="L49">
+        <f t="shared" si="2"/>
         <v>9.9274942592156024E-3</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M49">
+        <f t="shared" si="1"/>
+        <v>1.0003554609060716E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>0.4</v>
       </c>
@@ -1841,12 +2148,19 @@
       <c r="H50">
         <v>0.16486698568866401</v>
       </c>
-      <c r="J50">
-        <f t="shared" si="0"/>
+      <c r="I50">
+        <v>0.16703282909233391</v>
+      </c>
+      <c r="L50">
+        <f t="shared" si="2"/>
         <v>1.9675519311335987E-2</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M50">
+        <f t="shared" si="1"/>
+        <v>1.7509675907666084E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>0.3</v>
       </c>
@@ -1871,12 +2185,19 @@
       <c r="H51">
         <v>0.38736992880624621</v>
       </c>
-      <c r="J51">
-        <f t="shared" si="0"/>
+      <c r="I51">
+        <v>0.38960845651612108</v>
+      </c>
+      <c r="L51">
+        <f t="shared" si="2"/>
         <v>1.0964137193753776E-2</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M51">
+        <f t="shared" si="1"/>
+        <v>8.7256094838789044E-3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>0.3</v>
       </c>
@@ -1901,12 +2222,19 @@
       <c r="H52">
         <v>0.27975209158680281</v>
       </c>
-      <c r="J52">
-        <f t="shared" si="0"/>
+      <c r="I52">
+        <v>0.27784958903014301</v>
+      </c>
+      <c r="L52">
+        <f t="shared" si="2"/>
         <v>1.0164661413197218E-2</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M52">
+        <f t="shared" si="1"/>
+        <v>1.206716396985702E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>0.3</v>
       </c>
@@ -1931,12 +2259,19 @@
       <c r="H53">
         <v>0.2047464153679239</v>
       </c>
-      <c r="J53">
-        <f t="shared" si="0"/>
+      <c r="I53">
+        <v>0.20331655022203901</v>
+      </c>
+      <c r="L53">
+        <f t="shared" si="2"/>
         <v>1.3570548632076102E-2</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M53">
+        <f t="shared" si="1"/>
+        <v>1.5000413777960991E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>0.3</v>
       </c>
@@ -1961,12 +2296,19 @@
       <c r="H54">
         <v>0.15281640666452639</v>
       </c>
-      <c r="J54">
-        <f t="shared" si="0"/>
+      <c r="I54">
+        <v>0.15276152668377529</v>
+      </c>
+      <c r="L54">
+        <f t="shared" si="2"/>
         <v>3.1001190335473605E-2</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M54">
+        <f t="shared" si="1"/>
+        <v>3.1056070316224704E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>0.2</v>
       </c>
@@ -1991,12 +2333,19 @@
       <c r="H55">
         <v>0.36095215772374178</v>
       </c>
-      <c r="J55">
-        <f t="shared" si="0"/>
+      <c r="I55">
+        <v>0.36108169411581742</v>
+      </c>
+      <c r="L55">
+        <f t="shared" si="2"/>
         <v>2.13184492762582E-2</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M55">
+        <f t="shared" si="1"/>
+        <v>2.1188912884182565E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>0.2</v>
       </c>
@@ -2021,12 +2370,19 @@
       <c r="H56">
         <v>0.25952972987745832</v>
       </c>
-      <c r="J56">
-        <f t="shared" si="0"/>
+      <c r="I56">
+        <v>0.2590460610332494</v>
+      </c>
+      <c r="L56">
+        <f t="shared" si="2"/>
         <v>2.5501022122541683E-2</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M56">
+        <f t="shared" si="1"/>
+        <v>2.5984690966750601E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>0.2</v>
       </c>
@@ -2051,12 +2407,19 @@
       <c r="H57">
         <v>0.18666406157594351</v>
       </c>
-      <c r="J57">
-        <f t="shared" si="0"/>
+      <c r="I57">
+        <v>0.18704221993445219</v>
+      </c>
+      <c r="L57">
+        <f t="shared" si="2"/>
         <v>3.0287010424056487E-2</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M57">
+        <f t="shared" si="1"/>
+        <v>2.9908852065547803E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>0.2</v>
       </c>
@@ -2081,12 +2444,19 @@
       <c r="H58">
         <v>0.1267086052292109</v>
       </c>
-      <c r="J58">
-        <f t="shared" si="0"/>
+      <c r="I58">
+        <v>0.1270702709357717</v>
+      </c>
+      <c r="L58">
+        <f t="shared" si="2"/>
         <v>5.6739622770789089E-2</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M58">
+        <f t="shared" si="1"/>
+        <v>5.6377957064228296E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>0.1</v>
       </c>
@@ -2111,12 +2481,19 @@
       <c r="H59">
         <v>0.31959010294219647</v>
       </c>
-      <c r="J59">
-        <f t="shared" si="0"/>
+      <c r="I59">
+        <v>0.32007630972513518</v>
+      </c>
+      <c r="L59">
+        <f t="shared" si="2"/>
         <v>4.9625013057803535E-2</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M59">
+        <f t="shared" si="1"/>
+        <v>4.9138806274864832E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>0.1</v>
       </c>
@@ -2141,12 +2518,19 @@
       <c r="H60">
         <v>0.22220693884618539</v>
       </c>
-      <c r="J60">
-        <f t="shared" si="0"/>
+      <c r="I60">
+        <v>0.2212253719183446</v>
+      </c>
+      <c r="L60">
+        <f t="shared" si="2"/>
         <v>5.5356034153814598E-2</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M60">
+        <f t="shared" si="1"/>
+        <v>5.6337601081655392E-2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>0.1</v>
       </c>
@@ -2171,12 +2555,19 @@
       <c r="H61">
         <v>0.14475575445022701</v>
       </c>
-      <c r="J61">
-        <f t="shared" si="0"/>
+      <c r="I61">
+        <v>0.1444262488442998</v>
+      </c>
+      <c r="L61">
+        <f t="shared" si="2"/>
         <v>7.0463875549772986E-2</v>
       </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M61">
+        <f t="shared" si="1"/>
+        <v>7.0793381155700191E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>0.1</v>
       </c>
@@ -2201,12 +2592,19 @@
       <c r="H62">
         <v>8.7771304256109503E-2</v>
       </c>
-      <c r="J62">
-        <f t="shared" si="0"/>
+      <c r="I62">
+        <v>8.6428914543256088E-2</v>
+      </c>
+      <c r="L62">
+        <f t="shared" si="2"/>
         <v>9.486880874389049E-2</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M62">
+        <f t="shared" si="1"/>
+        <v>9.6211198456743904E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>0</v>
       </c>
@@ -2231,12 +2629,19 @@
       <c r="H63">
         <v>0.35560817910520681</v>
       </c>
-      <c r="J63">
-        <f t="shared" si="0"/>
+      <c r="I63">
+        <v>0.35675226295496137</v>
+      </c>
+      <c r="L63">
+        <f t="shared" si="2"/>
         <v>3.340828947931973E-4</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M63">
+        <f t="shared" si="1"/>
+        <v>-8.1000095496136515E-4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>0</v>
       </c>
@@ -2261,12 +2666,19 @@
       <c r="H64">
         <v>0.27205648857050557</v>
       </c>
-      <c r="J64">
-        <f t="shared" si="0"/>
+      <c r="I64">
+        <v>0.27157707945253162</v>
+      </c>
+      <c r="L64">
+        <f t="shared" si="2"/>
         <v>-5.1888257050558551E-4</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M64">
+        <f t="shared" si="1"/>
+        <v>-3.9473452531635367E-5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>0</v>
       </c>
@@ -2291,12 +2703,19 @@
       <c r="H65">
         <v>0.21306409487526101</v>
       </c>
-      <c r="J65">
-        <f t="shared" si="0"/>
+      <c r="I65">
+        <v>0.21319881139128311</v>
+      </c>
+      <c r="L65">
+        <f t="shared" si="2"/>
         <v>-2.5067887526100674E-4</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M65">
+        <f t="shared" si="1"/>
+        <v>-3.8539539128309985E-4</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>0</v>
       </c>
@@ -2321,9 +2740,16 @@
       <c r="H66">
         <v>0.18211015495034849</v>
       </c>
-      <c r="J66">
-        <f t="shared" si="0"/>
+      <c r="I66">
+        <v>0.1818487589063037</v>
+      </c>
+      <c r="L66">
+        <f t="shared" si="2"/>
         <v>1.015631049651522E-3</v>
+      </c>
+      <c r="M66">
+        <f t="shared" si="1"/>
+        <v>1.2770270936963146E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>